<commit_message>
Added new RDF data schemes and visual schemes for environment-table26-30, and fixed XLSX spreadsheets for environment-table26-30
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table26.xlsx
+++ b/sources/table_normalization/xlsx/environment-table26.xlsx
@@ -352,7 +352,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -453,7 +453,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -466,6 +465,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -775,7 +778,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1102,19 +1105,19 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="51" t="s">
+      <c r="B5" s="55"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="50" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="70">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="51" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -1650,7 +1653,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="18">
-      <c r="A25" s="53" t="s">
+      <c r="A25" s="52" t="s">
         <v>33</v>
       </c>
       <c r="B25" s="31">
@@ -1687,7 +1690,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="17.5">
-      <c r="A26" s="54" t="s">
+      <c r="A26" s="53" t="s">
         <v>34</v>
       </c>
       <c r="B26" s="33">
@@ -1724,7 +1727,7 @@
       </c>
     </row>
     <row r="27" spans="1:9" ht="17.5">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="53" t="s">
         <v>35</v>
       </c>
       <c r="B27" s="34">
@@ -1760,7 +1763,7 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="17.5">
-      <c r="A28" s="54" t="s">
+      <c r="A28" s="53" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="36">
@@ -1797,7 +1800,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="17.5">
-      <c r="A29" s="55" t="s">
+      <c r="A29" s="54" t="s">
         <v>38</v>
       </c>
       <c r="B29" s="33">

</xml_diff>